<commit_message>
data: monthly agent tally 2026-07-08
</commit_message>
<xml_diff>
--- a/COMP_Agent)Tally.xlsx
+++ b/COMP_Agent)Tally.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By State" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Market" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="By State" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="By Market" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>

</xml_diff>